<commit_message>
manual production scheduling changes
</commit_message>
<xml_diff>
--- a/outputs/simple-change-tracker/Factory_OS_Simple_Change_Tracker.xlsx
+++ b/outputs/simple-change-tracker/Factory_OS_Simple_Change_Tracker.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/diyaroongta/Downloads/factory-os/outputs/simple-change-tracker/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00098702-F806-444E-879D-5D6307223708}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A153706F-408E-DB4B-902B-89E0E68802B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17700" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="6700" yWindow="660" windowWidth="23540" windowHeight="17680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Changes" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
     <author>tc={E8971F82-44BE-9049-B9A9-3542313EFB10}</author>
   </authors>
   <commentList>
-    <comment ref="D8" authorId="0" shapeId="0" xr:uid="{E8971F82-44BE-9049-B9A9-3542313EFB10}">
+    <comment ref="D11" authorId="0" shapeId="0" xr:uid="{E8971F82-44BE-9049-B9A9-3542313EFB10}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="199" uniqueCount="69">
   <si>
     <t>Changes discussed</t>
   </si>
@@ -233,13 +233,25 @@
   </si>
   <si>
     <t>24th Aug</t>
+  </si>
+  <si>
+    <t>26th Aug</t>
+  </si>
+  <si>
+    <t>Order dispatch not linked to other tabs</t>
+  </si>
+  <si>
+    <t>PI database tab errors - ability to delete, sync across tabs, etc.</t>
+  </si>
+  <si>
+    <t>PI generation tab was wrong - reading sizing wrong, not able to edit PI blanks</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5">
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <name val="Carlito"/>
@@ -258,12 +270,6 @@
     <font>
       <sz val="8"/>
       <name val="Carlito"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Tahoma"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="6">
@@ -571,7 +577,7 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <threadedComment ref="D8" dT="2026-08-27T06:50:27.77" personId="{147206EA-79DD-7E49-ACCF-8E8B7C59AE3A}" id="{E8971F82-44BE-9049-B9A9-3542313EFB10}">
+  <threadedComment ref="D11" dT="2026-08-27T06:50:27.77" personId="{147206EA-79DD-7E49-ACCF-8E8B7C59AE3A}" id="{E8971F82-44BE-9049-B9A9-3542313EFB10}">
     <text>Due to model bugs</text>
   </threadedComment>
 </ThreadedComments>
@@ -579,7 +585,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D56"/>
+  <dimension ref="A1:D59"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
   <cols>
     <col min="2" max="2" width="64" customWidth="1"/>
@@ -600,12 +606,12 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="23" customHeight="1">
+    <row r="2" spans="1:4" ht="26" customHeight="1">
       <c r="A2" t="s">
-        <v>56</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>60</v>
+        <v>65</v>
+      </c>
+      <c r="B2" t="s">
+        <v>68</v>
       </c>
       <c r="C2" s="6" t="s">
         <v>4</v>
@@ -614,12 +620,12 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="23" customHeight="1">
+    <row r="3" spans="1:4" ht="26" customHeight="1">
       <c r="A3" t="s">
-        <v>56</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>62</v>
+        <v>65</v>
+      </c>
+      <c r="B3" t="s">
+        <v>66</v>
       </c>
       <c r="C3" s="6" t="s">
         <v>4</v>
@@ -628,12 +634,12 @@
         <v>25</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="23" customHeight="1">
+    <row r="4" spans="1:4" ht="26" customHeight="1">
       <c r="A4" t="s">
-        <v>56</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>61</v>
+        <v>65</v>
+      </c>
+      <c r="B4" t="s">
+        <v>67</v>
       </c>
       <c r="C4" s="6" t="s">
         <v>4</v>
@@ -647,7 +653,7 @@
         <v>56</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>3</v>
+        <v>60</v>
       </c>
       <c r="C5" s="6" t="s">
         <v>4</v>
@@ -661,7 +667,7 @@
         <v>56</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>6</v>
+        <v>62</v>
       </c>
       <c r="C6" s="6" t="s">
         <v>4</v>
@@ -675,7 +681,7 @@
         <v>56</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>7</v>
+        <v>61</v>
       </c>
       <c r="C7" s="6" t="s">
         <v>4</v>
@@ -689,13 +695,13 @@
         <v>56</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="C8" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>5</v>
+        <v>3</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="D8" s="8" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="23" customHeight="1">
@@ -703,27 +709,27 @@
         <v>56</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="C9" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="D9" s="4" t="s">
-        <v>5</v>
+        <v>6</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="D9" s="8" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="23" customHeight="1">
       <c r="A10" t="s">
-        <v>64</v>
+        <v>56</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="C10" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="D10" s="4" t="s">
-        <v>5</v>
+        <v>7</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="D10" s="8" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="23" customHeight="1">
@@ -731,7 +737,7 @@
         <v>56</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>8</v>
+        <v>59</v>
       </c>
       <c r="C11" s="7" t="s">
         <v>9</v>
@@ -745,10 +751,10 @@
         <v>56</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="C12" s="6" t="s">
-        <v>4</v>
+        <v>58</v>
+      </c>
+      <c r="C12" s="7" t="s">
+        <v>9</v>
       </c>
       <c r="D12" s="4" t="s">
         <v>5</v>
@@ -756,16 +762,16 @@
     </row>
     <row r="13" spans="1:4" ht="23" customHeight="1">
       <c r="A13" t="s">
-        <v>56</v>
+        <v>64</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C13" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="D13" s="8" t="s">
-        <v>25</v>
+        <v>63</v>
+      </c>
+      <c r="C13" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="23" customHeight="1">
@@ -773,13 +779,13 @@
         <v>56</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C14" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="D14" s="8" t="s">
-        <v>25</v>
+        <v>8</v>
+      </c>
+      <c r="C14" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="23" customHeight="1">
@@ -787,13 +793,13 @@
         <v>56</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="C15" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="D15" s="8" t="s">
-        <v>25</v>
+      <c r="D15" s="4" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="23" customHeight="1">
@@ -801,13 +807,13 @@
         <v>56</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="C16" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="D16" s="4" t="s">
-        <v>5</v>
+      <c r="D16" s="8" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="23" customHeight="1">
@@ -815,13 +821,13 @@
         <v>56</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="C17" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="D17" s="4" t="s">
-        <v>5</v>
+      <c r="D17" s="8" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="18" spans="1:4" ht="23" customHeight="1">
@@ -829,13 +835,13 @@
         <v>56</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="C18" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="D18" s="4" t="s">
-        <v>5</v>
+      <c r="D18" s="8" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="23" customHeight="1">
@@ -843,7 +849,7 @@
         <v>56</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="C19" s="6" t="s">
         <v>4</v>
@@ -857,7 +863,7 @@
         <v>56</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="C20" s="6" t="s">
         <v>4</v>
@@ -871,7 +877,7 @@
         <v>56</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="C21" s="6" t="s">
         <v>4</v>
@@ -882,57 +888,66 @@
     </row>
     <row r="22" spans="1:4" ht="23" customHeight="1">
       <c r="A22" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="C22" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C22" s="6" t="s">
         <v>4</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>25</v>
+        <v>5</v>
       </c>
     </row>
     <row r="23" spans="1:4" ht="23" customHeight="1">
       <c r="A23" t="s">
+        <v>56</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C23" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="D23" s="4" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" ht="23" customHeight="1">
+      <c r="A24" t="s">
+        <v>56</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C24" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="D24" s="4" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" ht="23" customHeight="1">
+      <c r="A25" t="s">
         <v>57</v>
       </c>
-      <c r="B23" s="2" t="s">
+      <c r="B25" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D25" s="4" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" ht="23" customHeight="1">
+      <c r="A26" t="s">
+        <v>57</v>
+      </c>
+      <c r="B26" s="2" t="s">
         <v>20</v>
-      </c>
-      <c r="C23" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="D23" s="4" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" ht="23" customHeight="1">
-      <c r="B24" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="C24" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="D24" s="4" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" ht="23" customHeight="1">
-      <c r="B25" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="C25" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="D25" s="4" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" ht="23" customHeight="1">
-      <c r="B26" s="2" t="s">
-        <v>23</v>
       </c>
       <c r="C26" s="4" t="s">
         <v>4</v>
@@ -943,7 +958,7 @@
     </row>
     <row r="27" spans="1:4" ht="23" customHeight="1">
       <c r="B27" s="2" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="C27" s="4" t="s">
         <v>4</v>
@@ -954,7 +969,7 @@
     </row>
     <row r="28" spans="1:4" ht="23" customHeight="1">
       <c r="B28" s="2" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="C28" s="4" t="s">
         <v>4</v>
@@ -965,7 +980,7 @@
     </row>
     <row r="29" spans="1:4" ht="23" customHeight="1">
       <c r="B29" s="2" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="C29" s="4" t="s">
         <v>4</v>
@@ -976,7 +991,7 @@
     </row>
     <row r="30" spans="1:4" ht="23" customHeight="1">
       <c r="B30" s="2" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="C30" s="4" t="s">
         <v>4</v>
@@ -987,7 +1002,7 @@
     </row>
     <row r="31" spans="1:4" ht="23" customHeight="1">
       <c r="B31" s="2" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="C31" s="4" t="s">
         <v>4</v>
@@ -998,7 +1013,7 @@
     </row>
     <row r="32" spans="1:4" ht="23" customHeight="1">
       <c r="B32" s="2" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="C32" s="4" t="s">
         <v>4</v>
@@ -1009,7 +1024,7 @@
     </row>
     <row r="33" spans="2:4" ht="23" customHeight="1">
       <c r="B33" s="2" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="C33" s="4" t="s">
         <v>4</v>
@@ -1020,7 +1035,7 @@
     </row>
     <row r="34" spans="2:4" ht="23" customHeight="1">
       <c r="B34" s="2" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="C34" s="4" t="s">
         <v>4</v>
@@ -1031,7 +1046,7 @@
     </row>
     <row r="35" spans="2:4" ht="23" customHeight="1">
       <c r="B35" s="2" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="C35" s="4" t="s">
         <v>4</v>
@@ -1042,7 +1057,7 @@
     </row>
     <row r="36" spans="2:4" ht="23" customHeight="1">
       <c r="B36" s="2" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C36" s="4" t="s">
         <v>4</v>
@@ -1053,7 +1068,7 @@
     </row>
     <row r="37" spans="2:4" ht="23" customHeight="1">
       <c r="B37" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="C37" s="4" t="s">
         <v>4</v>
@@ -1064,7 +1079,7 @@
     </row>
     <row r="38" spans="2:4" ht="23" customHeight="1">
       <c r="B38" s="2" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="C38" s="4" t="s">
         <v>4</v>
@@ -1075,7 +1090,7 @@
     </row>
     <row r="39" spans="2:4" ht="23" customHeight="1">
       <c r="B39" s="2" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="C39" s="4" t="s">
         <v>4</v>
@@ -1086,7 +1101,7 @@
     </row>
     <row r="40" spans="2:4" ht="23" customHeight="1">
       <c r="B40" s="2" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="C40" s="4" t="s">
         <v>4</v>
@@ -1097,7 +1112,7 @@
     </row>
     <row r="41" spans="2:4" ht="23" customHeight="1">
       <c r="B41" s="2" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="C41" s="4" t="s">
         <v>4</v>
@@ -1108,7 +1123,7 @@
     </row>
     <row r="42" spans="2:4" ht="23" customHeight="1">
       <c r="B42" s="2" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="C42" s="4" t="s">
         <v>4</v>
@@ -1119,7 +1134,7 @@
     </row>
     <row r="43" spans="2:4" ht="23" customHeight="1">
       <c r="B43" s="2" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="C43" s="4" t="s">
         <v>4</v>
@@ -1130,7 +1145,7 @@
     </row>
     <row r="44" spans="2:4" ht="23" customHeight="1">
       <c r="B44" s="2" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="C44" s="4" t="s">
         <v>4</v>
@@ -1141,7 +1156,7 @@
     </row>
     <row r="45" spans="2:4" ht="23" customHeight="1">
       <c r="B45" s="2" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="C45" s="4" t="s">
         <v>4</v>
@@ -1152,7 +1167,7 @@
     </row>
     <row r="46" spans="2:4" ht="23" customHeight="1">
       <c r="B46" s="2" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="C46" s="4" t="s">
         <v>4</v>
@@ -1163,7 +1178,7 @@
     </row>
     <row r="47" spans="2:4" ht="23" customHeight="1">
       <c r="B47" s="2" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="C47" s="4" t="s">
         <v>4</v>
@@ -1174,7 +1189,7 @@
     </row>
     <row r="48" spans="2:4" ht="23" customHeight="1">
       <c r="B48" s="2" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="C48" s="4" t="s">
         <v>4</v>
@@ -1185,7 +1200,7 @@
     </row>
     <row r="49" spans="2:4" ht="23" customHeight="1">
       <c r="B49" s="2" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="C49" s="4" t="s">
         <v>4</v>
@@ -1196,7 +1211,7 @@
     </row>
     <row r="50" spans="2:4" ht="23" customHeight="1">
       <c r="B50" s="2" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="C50" s="4" t="s">
         <v>4</v>
@@ -1207,7 +1222,7 @@
     </row>
     <row r="51" spans="2:4" ht="23" customHeight="1">
       <c r="B51" s="2" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="C51" s="4" t="s">
         <v>4</v>
@@ -1218,7 +1233,7 @@
     </row>
     <row r="52" spans="2:4" ht="23" customHeight="1">
       <c r="B52" s="2" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="C52" s="4" t="s">
         <v>4</v>
@@ -1229,7 +1244,7 @@
     </row>
     <row r="53" spans="2:4" ht="23" customHeight="1">
       <c r="B53" s="2" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="C53" s="4" t="s">
         <v>4</v>
@@ -1240,32 +1255,65 @@
     </row>
     <row r="54" spans="2:4" ht="23" customHeight="1">
       <c r="B54" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C54" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D54" s="4" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="55" spans="2:4" ht="23" customHeight="1">
+      <c r="B55" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="C55" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D55" s="4" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="56" spans="2:4" ht="23" customHeight="1">
+      <c r="B56" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="C56" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D56" s="4" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="57" spans="2:4" ht="23" customHeight="1">
+      <c r="B57" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="C54" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="D54" s="5" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="55" spans="2:4">
-      <c r="B55" s="2" t="s">
+      <c r="C57" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="D57" s="5" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="58" spans="2:4">
+      <c r="B58" s="2" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="56" spans="2:4">
-      <c r="B56" s="3" t="s">
+    <row r="59" spans="2:4">
+      <c r="B59" s="3" t="s">
         <v>54</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
   <dataValidations count="2">
-    <dataValidation type="list" sqref="C2:C54" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" sqref="C2:C57" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Abhay,Diya"</formula1>
     </dataValidation>
-    <dataValidation type="list" sqref="D2:D54" xr:uid="{00000000-0002-0000-0000-000001000000}">
+    <dataValidation type="list" sqref="D2:D57" xr:uid="{00000000-0002-0000-0000-000001000000}">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>